<commit_message>
fix: repair broken site report formulas
</commit_message>
<xml_diff>
--- a/attachments/TheCapitol_MSK_Report.xlsx
+++ b/attachments/TheCapitol_MSK_Report.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alvin\Desktop\GM\reports\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C4ADF3-3FB4-431D-9695-D1BCF026F731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="C:\Users\alvin\Desktop\GM\reports\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C4ADF3-3FB4-431D-9695-D1BCF026F731}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" ns6:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PROGRESSION" sheetId="1" r:id="rId1"/>
-    <sheet name="COMPARE" sheetId="4" r:id="rId2"/>
-    <sheet name="ORDER" sheetId="6" r:id="rId3"/>
-    <sheet name="FLOORS" sheetId="5" r:id="rId4"/>
-    <sheet name="SITE REPORT" sheetId="7" r:id="rId5"/>
-    <sheet name="PO LOG" sheetId="8" r:id="rId6"/>
-    <sheet name="MANPOWER" sheetId="9" r:id="rId7"/>
-    <sheet name="ATTENDANCE" sheetId="12" r:id="rId8"/>
-    <sheet name="aipoon" sheetId="15" r:id="rId9"/>
-    <sheet name="ariyan" sheetId="16" r:id="rId10"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId11"/>
+    <sheet name="PROGRESSION" sheetId="1" ns7:id="rId1"/>
+    <sheet name="COMPARE" sheetId="4" ns7:id="rId2"/>
+    <sheet name="ORDER" sheetId="6" ns7:id="rId3"/>
+    <sheet name="FLOORS" sheetId="5" ns7:id="rId4"/>
+    <sheet name="SITE REPORT" sheetId="7" ns7:id="rId5"/>
+    <sheet name="PO LOG" sheetId="8" ns7:id="rId6"/>
+    <sheet name="MANPOWER" sheetId="9" ns7:id="rId7"/>
+    <sheet name="ATTENDANCE" sheetId="12" ns7:id="rId8"/>
+    <sheet name="aipoon" sheetId="15" ns7:id="rId9"/>
+    <sheet name="ariyan" sheetId="16" ns7:id="rId10"/>
+    <sheet name="Sheet2" sheetId="3" ns7:id="rId11"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId12"/>
+    <externalReference ns7:id="rId12"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="7">ATTENDANCE!$A$1:$AF$28</definedName>
@@ -35,18 +35,18 @@
     <definedName name="solver_eng" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_eng" localSheetId="4" hidden="1">0</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns8:calcFeatures>
+        <ns8:feature name="microsoft.com:RD"/>
+        <ns8:feature name="microsoft.com:Single"/>
+        <ns8:feature name="microsoft.com:FV"/>
+        <ns8:feature name="microsoft.com:CNMTM"/>
+        <ns8:feature name="microsoft.com:LET_WF"/>
+        <ns8:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns8:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns8:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -9032,7 +9032,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AK46"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
@@ -9081,9 +9081,6 @@
       <c r="O1" s="119"/>
       <c r="P1" s="119"/>
       <c r="Q1" s="119"/>
-      <c r="R1" s="109" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="2" spans="1:27" s="16" customFormat="1" ht="36.6">
       <c r="A2" s="120" t="s">
@@ -11431,8 +11428,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3B394AC6-2E33-4111-9224-3A1DE849EBEE}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{3B394AC6-2E33-4111-9224-3A1DE849EBEE}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11455,8 +11452,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1B66B904-3451-4A48-A042-72A3E9767670}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{1B66B904-3451-4A48-A042-72A3E9767670}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11489,8 +11486,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6178F2FF-113A-4D64-9A55-F806E0F38586}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{6178F2FF-113A-4D64-9A55-F806E0F38586}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11503,8 +11500,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E75B804D-4D4B-4159-994A-4DC4901D3238}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{E75B804D-4D4B-4159-994A-4DC4901D3238}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11539,8 +11536,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3FD3A52A-BC28-4A5A-A370-5A406081130B}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{3FD3A52A-BC28-4A5A-A370-5A406081130B}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11563,8 +11560,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FEDFC549-DCEE-43AB-8AEE-02765F872CA2}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{FEDFC549-DCEE-43AB-8AEE-02765F872CA2}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11598,8 +11595,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5BD8B6D8-4968-4DD8-B8A9-471FEAEE192A}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{5BD8B6D8-4968-4DD8-B8A9-471FEAEE192A}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11612,8 +11609,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{96641237-F530-4C30-923D-98375C20AC04}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{96641237-F530-4C30-923D-98375C20AC04}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11646,8 +11643,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A8162A29-376F-4F8E-A008-69A52B3FC97F}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{A8162A29-376F-4F8E-A008-69A52B3FC97F}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11670,8 +11667,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2B457CDA-192A-498B-B097-84F5697D58BB}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{2B457CDA-192A-498B-B097-84F5697D58BB}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11684,8 +11681,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{00B6732A-CE6C-476A-8627-02916E2796BE}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{00B6732A-CE6C-476A-8627-02916E2796BE}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11706,8 +11703,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{344FFAF0-A7F2-4DB5-8C70-5C08C1A6FCD1}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{344FFAF0-A7F2-4DB5-8C70-5C08C1A6FCD1}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11730,8 +11727,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{43AF006F-A636-4326-9F07-36CABC7C1F74}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{43AF006F-A636-4326-9F07-36CABC7C1F74}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11764,8 +11761,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95524A12-9B14-4609-939A-715A879D0E52}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{95524A12-9B14-4609-939A-715A879D0E52}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11788,8 +11785,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BBC338D7-3AFD-45D1-A161-34D342C18D75}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{BBC338D7-3AFD-45D1-A161-34D342C18D75}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11812,8 +11809,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6C6F3769-45B6-4FEF-BF4B-2C3B277227D8}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{6C6F3769-45B6-4FEF-BF4B-2C3B277227D8}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11836,8 +11833,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BFCCFE2F-14AB-4A3E-99DF-3961DC7B0CDB}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{BFCCFE2F-14AB-4A3E-99DF-3961DC7B0CDB}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11858,8 +11855,8 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CA285D16-D2E2-487F-9BBB-9F9D79273182}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{CA285D16-D2E2-487F-9BBB-9F9D79273182}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11882,221 +11879,221 @@
         <color rgb="FF63C384"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C5AC0648-6C1E-4510-BA28-776FAAE3221F}</x14:id>
+        <ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns3:id>{C5AC0648-6C1E-4510-BA28-776FAAE3221F}</ns3:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" ns4:id="rId1"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3B394AC6-2E33-4111-9224-3A1DE849EBEE}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C6:C25 F6:R6 F24:M25 J34:L35 F44:L45 C45 N25:R25 N34:Q44 N45:R45 N15:R16 N17:Q24 L6:L25 L36:L45 F7:F23 N7:Q14 F33:F43 H26:H41 H7:M23 H36:L43</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1B66B904-3451-4A48-A042-72A3E9767670}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C6:C25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6178F2FF-113A-4D64-9A55-F806E0F38586}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C6:C45 F6:R45</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E75B804D-4D4B-4159-994A-4DC4901D3238}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C26:C44</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3FD3A52A-BC28-4A5A-A370-5A406081130B}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C27:C43 C26 C44</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FEDFC549-DCEE-43AB-8AEE-02765F872CA2}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C6:R45</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5BD8B6D8-4968-4DD8-B8A9-471FEAEE192A}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D6:E6 D24:E25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{96641237-F530-4C30-923D-98375C20AC04}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D6:E25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A8162A29-376F-4F8E-A008-69A52B3FC97F}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D26:E26 D44:E45</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2B457CDA-192A-498B-B097-84F5697D58BB}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D26:E45</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{00B6732A-CE6C-476A-8627-02916E2796BE}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <x14:cfRule type="dataBar" id="{344FFAF0-A7F2-4DB5-8C70-5C08C1A6FCD1}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>F26:F43</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{43AF006F-A636-4326-9F07-36CABC7C1F74}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>G26</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95524A12-9B14-4609-939A-715A879D0E52}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>I26:I35</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BBC338D7-3AFD-45D1-A161-34D342C18D75}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>J34:K35 J26:Q33 M28:M36</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6C6F3769-45B6-4FEF-BF4B-2C3B277227D8}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>L26:L35</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BFCCFE2F-14AB-4A3E-99DF-3961DC7B0CDB}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <x14:cfRule type="dataBar" id="{CA285D16-D2E2-487F-9BBB-9F9D79273182}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>M34:M45</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C5AC0648-6C1E-4510-BA28-776FAAE3221F}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>R35:R36 R26</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
+    <ext uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <ns3:conditionalFormattings>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{3B394AC6-2E33-4111-9224-3A1DE849EBEE}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>C6:C25 F6:R6 F24:M25 J34:L35 F44:L45 C45 N25:R25 N34:Q44 N45:R45 N15:R16 N17:Q24 L6:L25 L36:L45 F7:F23 N7:Q14 F33:F43 H26:H41 H7:M23 H36:L43</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{1B66B904-3451-4A48-A042-72A3E9767670}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>C6:C25</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{6178F2FF-113A-4D64-9A55-F806E0F38586}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>C6:C45 F6:R45</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{E75B804D-4D4B-4159-994A-4DC4901D3238}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>C26:C44</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{3FD3A52A-BC28-4A5A-A370-5A406081130B}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>C27:C43 C26 C44</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{FEDFC549-DCEE-43AB-8AEE-02765F872CA2}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>C6:R45</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{5BD8B6D8-4968-4DD8-B8A9-471FEAEE192A}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>D6:E6 D24:E25</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{96641237-F530-4C30-923D-98375C20AC04}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>D6:E25</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{A8162A29-376F-4F8E-A008-69A52B3FC97F}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>D26:E26 D44:E45</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{2B457CDA-192A-498B-B097-84F5697D58BB}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>D26:E45</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{00B6732A-CE6C-476A-8627-02916E2796BE}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns3:cfRule type="dataBar" id="{344FFAF0-A7F2-4DB5-8C70-5C08C1A6FCD1}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>F26:F43</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{43AF006F-A636-4326-9F07-36CABC7C1F74}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>G26</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{95524A12-9B14-4609-939A-715A879D0E52}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>I26:I35</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{BBC338D7-3AFD-45D1-A161-34D342C18D75}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>J34:K35 J26:Q33 M28:M36</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{6C6F3769-45B6-4FEF-BF4B-2C3B277227D8}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>L26:L35</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{BFCCFE2F-14AB-4A3E-99DF-3961DC7B0CDB}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns3:cfRule type="dataBar" id="{CA285D16-D2E2-487F-9BBB-9F9D79273182}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>M34:M45</ns5:sqref>
+        </ns3:conditionalFormatting>
+        <ns3:conditionalFormatting>
+          <ns3:cfRule type="dataBar" id="{C5AC0648-6C1E-4510-BA28-776FAAE3221F}">
+            <ns3:dataBar minLength="0" maxLength="100" gradient="0">
+              <ns3:cfvo type="autoMin"/>
+              <ns3:cfvo type="autoMax"/>
+              <ns3:negativeFillColor rgb="FFFF0000"/>
+              <ns3:axisColor rgb="FF000000"/>
+            </ns3:dataBar>
+          </ns3:cfRule>
+          <ns5:sqref>R35:R36 R26</ns5:sqref>
+        </ns3:conditionalFormatting>
+      </ns3:conditionalFormattings>
     </ext>
   </extLst>
 </worksheet>
@@ -15781,7 +15778,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AF2B2D8-7B23-4DF8-A9D4-0715BAC2C977}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{5AF2B2D8-7B23-4DF8-A9D4-0715BAC2C977}">
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
@@ -15920,310 +15917,250 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B13" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C13" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D13" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A13" s="50" t="str">
+        <f>PROGRESSION!C$5</f>
+        <v>PIPE SLEEVE</v>
+      </c>
+      <c r="B13" s="45">
+        <f>PROGRESSION!C$46</f>
+        <v>0.93125</v>
+      </c>
+      <c r="C13" s="50" t="str">
+        <f>IF(B13&gt;=0.9,"Complete",IF(B13&gt;0,"In Progress","Not Started"))</f>
+        <v>Complete</v>
+      </c>
+      <c r="D13" s="50"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B14" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C14" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D14" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A14" s="50" t="str">
+        <f>PROGRESSION!D$5</f>
+        <v>PUMP</v>
+      </c>
+      <c r="B14" s="45">
+        <f>PROGRESSION!D$46</f>
+        <v>0.475</v>
+      </c>
+      <c r="C14" s="50" t="str">
+        <f>IF(B14&gt;=0.9,"Complete",IF(B14&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D14" s="50"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B15" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C15" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D15" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A15" s="50" t="str">
+        <f>PROGRESSION!E$5</f>
+        <v>PUMP CONTROL PANEL</v>
+      </c>
+      <c r="B15" s="45">
+        <f>PROGRESSION!E$46</f>
+        <v>0.475</v>
+      </c>
+      <c r="C15" s="50" t="str">
+        <f>IF(B15&gt;=0.9,"Complete",IF(B15&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D15" s="50"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B16" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C16" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D16" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A16" s="50" t="str">
+        <f>PROGRESSION!F$5</f>
+        <v>TRANSFER PUMP PIPES</v>
+      </c>
+      <c r="B16" s="45">
+        <f>PROGRESSION!F$46</f>
+        <v>0.54625</v>
+      </c>
+      <c r="C16" s="50" t="str">
+        <f>IF(B16&gt;=0.9,"Complete",IF(B16&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D16" s="50"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B17" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C17" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D17" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A17" s="50" t="str">
+        <f>PROGRESSION!G$5</f>
+        <v>L31 &amp; 31M ROOF PIPING</v>
+      </c>
+      <c r="B17" s="45">
+        <f>PROGRESSION!G$46</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="50" t="str">
+        <f>IF(B17&gt;=0.9,"Complete",IF(B17&gt;0,"In Progress","Not Started"))</f>
+        <v>Not Started</v>
+      </c>
+      <c r="D17" s="50"/>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B18" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C18" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D18" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A18" s="50" t="str">
+        <f>PROGRESSION!H$5</f>
+        <v>CW TENANT</v>
+      </c>
+      <c r="B18" s="45">
+        <f>PROGRESSION!H$46</f>
+        <v>0.78375</v>
+      </c>
+      <c r="C18" s="50" t="str">
+        <f>IF(B18&gt;=0.9,"Complete",IF(B18&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D18" s="50"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B19" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C19" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D19" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A19" s="50" t="str">
+        <f>PROGRESSION!I$5</f>
+        <v>BACKSHAFT CW &amp; FW TOILETS</v>
+      </c>
+      <c r="B19" s="45">
+        <f>PROGRESSION!I$46</f>
+        <v>0.12125</v>
+      </c>
+      <c r="C19" s="50" t="str">
+        <f>IF(B19&gt;=0.9,"Complete",IF(B19&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D19" s="50"/>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B20" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C20" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D20" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A20" s="50" t="str">
+        <f>PROGRESSION!J$5</f>
+        <v>HOSEREEL FLOORTRAP &amp; STACK</v>
+      </c>
+      <c r="B20" s="45">
+        <f>PROGRESSION!J$46</f>
+        <v>0.5775</v>
+      </c>
+      <c r="C20" s="50" t="str">
+        <f>IF(B20&gt;=0.9,"Complete",IF(B20&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D20" s="50"/>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B21" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C21" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D21" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A21" s="50" t="str">
+        <f>PROGRESSION!K$5</f>
+        <v>SANITARY TENANT</v>
+      </c>
+      <c r="B21" s="45">
+        <f>PROGRESSION!K$46</f>
+        <v>0.5775</v>
+      </c>
+      <c r="C21" s="50" t="str">
+        <f>IF(B21&gt;=0.9,"Complete",IF(B21&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D21" s="50"/>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B22" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C22" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D22" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A22" s="50" t="str">
+        <f>PROGRESSION!L$5</f>
+        <v>TOILET PIPE DISTRIBUTION &amp; HACKING</v>
+      </c>
+      <c r="B22" s="45">
+        <f>PROGRESSION!L$46</f>
+        <v>0.395</v>
+      </c>
+      <c r="C22" s="50" t="str">
+        <f>IF(B22&gt;=0.9,"Complete",IF(B22&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D22" s="50"/>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B23" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C23" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D23" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A23" s="50" t="str">
+        <f>PROGRESSION!M$5</f>
+        <v>SANITARY TOILETS</v>
+      </c>
+      <c r="B23" s="45">
+        <f>PROGRESSION!M$46</f>
+        <v>0.65375</v>
+      </c>
+      <c r="C23" s="50" t="str">
+        <f>IF(B23&gt;=0.9,"Complete",IF(B23&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D23" s="50"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B24" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C24" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D24" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A24" s="50" t="str">
+        <f>PROGRESSION!N$5</f>
+        <v>SANITARY WARES INSTALLATION</v>
+      </c>
+      <c r="B24" s="45">
+        <f>PROGRESSION!N$46</f>
+        <v>0.1475</v>
+      </c>
+      <c r="C24" s="50" t="str">
+        <f>IF(B24&gt;=0.9,"Complete",IF(B24&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D24" s="50"/>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B25" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C25" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D25" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A25" s="50" t="str">
+        <f>PROGRESSION!O$5</f>
+        <v>IRRIGATION OUTLET</v>
+      </c>
+      <c r="B25" s="45">
+        <f>PROGRESSION!O$46</f>
+        <v>0.2</v>
+      </c>
+      <c r="C25" s="50" t="str">
+        <f>IF(B25&gt;=0.9,"Complete",IF(B25&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D25" s="50"/>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B26" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C26" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D26" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A26" s="50" t="str">
+        <f>PROGRESSION!P$5</f>
+        <v>IRRIGATION INLET</v>
+      </c>
+      <c r="B26" s="45">
+        <f>PROGRESSION!P$46</f>
+        <v>0.045</v>
+      </c>
+      <c r="C26" s="50" t="str">
+        <f>IF(B26&gt;=0.9,"Complete",IF(B26&gt;0,"In Progress","Not Started"))</f>
+        <v>In Progress</v>
+      </c>
+      <c r="D26" s="50"/>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B27" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C27" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D27" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A27" s="50" t="str">
+        <f>PROGRESSION!Q$5</f>
+        <v>IRRIGATION WIRING</v>
+      </c>
+      <c r="B27" s="45">
+        <f>PROGRESSION!Q$46</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="50" t="str">
+        <f>IF(B27&gt;=0.9,"Complete",IF(B27&gt;0,"In Progress","Not Started"))</f>
+        <v>Not Started</v>
+      </c>
+      <c r="D27" s="50"/>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B28" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C28" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D28" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A28" s="50" t="str">
+        <f>PROGRESSION!R$5</f>
+        <v>IRRIGATION CONTROL PANEL</v>
+      </c>
+      <c r="B28" s="45">
+        <f>PROGRESSION!R$46</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="50" t="str">
+        <f>IF(B28&gt;=0.9,"Complete",IF(B28&gt;0,"In Progress","Not Started"))</f>
+        <v>Not Started</v>
+      </c>
+      <c r="D28" s="50"/>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B29" s="45" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C29" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D29" s="50" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="A29" s="50"/>
+      <c r="B29" s="45"/>
+      <c r="C29" s="50"/>
+      <c r="D29" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -16245,8 +16182,8 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" ns3:id="rId1"/>
+  <drawing ns3:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>